<commit_message>
Refactor income calculation logic and update utility functions; enhance data processing in main script
</commit_message>
<xml_diff>
--- a/consolidado_exogena.xlsx
+++ b/consolidado_exogena.xlsx
@@ -1,76 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acuerdode-my.sharepoint.com/personal/sistemas_eso_gov_co/Documents/Preparador de exogenas/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_2B59F87F116F43CA216FC1925D1510344D07F0A2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E979B4F3-50EB-42D6-9700-875222382CB5}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Ingresos" sheetId="1" r:id="rId1"/>
+    <sheet name="Ingresos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>NIT Receptor</t>
-  </si>
-  <si>
-    <t>DV</t>
-  </si>
-  <si>
-    <t>Nombre Receptor</t>
-  </si>
-  <si>
-    <t>Base</t>
-  </si>
-  <si>
-    <t>IVA</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>LEONARDO MUÑOZ VELASQUEZ</t>
-  </si>
-  <si>
-    <t>CORPORACION COLEGIO NUEVA GRANADA</t>
-  </si>
-  <si>
-    <t>GRUPO GASTRONOMICO LA SEÑO SAS</t>
-  </si>
-  <si>
-    <t>ENTORNO CONSULTORIA, DISEÑO Y SERVICIOS AMBIENTALES SAS</t>
-  </si>
-  <si>
-    <t>EMPRESA DE DESARROLLO TERRITORIAL DE DONMATÍAS S.A.S.</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -89,21 +47,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -391,134 +408,131 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="3.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="59.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>NIT Receptor</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>DV</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Nombre Receptor</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>IVA</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>860006522</v>
+      </c>
+      <c r="B2" t="n">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CORPORACION COLEGIO NUEVA GRANADA</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1080000</v>
+      </c>
+      <c r="E2" t="n">
+        <v>205200</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1405200</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>901487993</v>
+      </c>
+      <c r="B3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GRUPO GASTRONOMICO LA SEÑO SAS</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>151260</v>
+      </c>
+      <c r="E3" t="n">
+        <v>28739.4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>179999</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>901551640</v>
+      </c>
+      <c r="B4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ENTORNO CONSULTORIA, DISEÑO Y SERVICIOS AMBIENTALES SAS</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>328947369.0526316</v>
+      </c>
+      <c r="E4" t="n">
+        <v>62500000.12</v>
+      </c>
+      <c r="F4" t="n">
+        <v>391447369</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>901852866</v>
+      </c>
+      <c r="B5" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>71774989</v>
-      </c>
-      <c r="B2">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>13332000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>860006522</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3">
-        <v>1080000</v>
-      </c>
-      <c r="E3">
-        <v>205200</v>
-      </c>
-      <c r="F3">
-        <v>1405200</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>901487993</v>
-      </c>
-      <c r="B4">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4">
-        <v>151260</v>
-      </c>
-      <c r="E4">
-        <v>28739.4</v>
-      </c>
-      <c r="F4">
-        <v>179999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>901551640</v>
-      </c>
-      <c r="B5">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5">
-        <v>328947369.05263162</v>
-      </c>
-      <c r="E5">
-        <v>62500000.119999997</v>
-      </c>
-      <c r="F5">
-        <v>391447369</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>901852866</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EMPRESA DE DESARROLLO TERRITORIAL DE DONMATÍAS S.A.S.</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
         <v>82845580</v>
       </c>
-      <c r="E6">
-        <v>15740660.199999999</v>
-      </c>
-      <c r="F6">
+      <c r="E5" t="n">
+        <v>15740660.2</v>
+      </c>
+      <c r="F5" t="n">
         <v>98586240</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add functionality to calculate and consolidate credit notes; update main script to process new data
</commit_message>
<xml_diff>
--- a/consolidado_exogena.xlsx
+++ b/consolidado_exogena.xlsx
@@ -1,34 +1,73 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acuerdode-my.sharepoint.com/personal/sistemas_eso_gov_co/Documents/Preparador de exogenas/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_2B59F87F11DFCA2F158BC0F34C1510344D07F1B2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB9CA89E-D6A6-4103-8034-104691F1B399}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Ingresos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ingresos" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>NIT Receptor</t>
+  </si>
+  <si>
+    <t>DV</t>
+  </si>
+  <si>
+    <t>Nombre Receptor</t>
+  </si>
+  <si>
+    <t>Base</t>
+  </si>
+  <si>
+    <t>IVA</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>CORPORACION COLEGIO NUEVA GRANADA</t>
+  </si>
+  <si>
+    <t>GRUPO GASTRONOMICO LA SEÑO SAS</t>
+  </si>
+  <si>
+    <t>ENTORNO CONSULTORIA, DISEÑO Y SERVICIOS AMBIENTALES SAS</t>
+  </si>
+  <si>
+    <t>EMPRESA DE DESARROLLO TERRITORIAL DE DONMATÍAS S.A.S.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,80 +86,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,131 +388,115 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Hoja1"/>
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="55.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>NIT Receptor</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>DV</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Nombre Receptor</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>IVA</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
         <v>860006522</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>0</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CORPORACION COLEGIO NUEVA GRANADA</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2">
         <v>1080000</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>205200</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>1405200</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
         <v>901487993</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3">
         <v>7</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GRUPO GASTRONOMICO LA SEÑO SAS</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
         <v>151260</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>28739.4</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>179999</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>901551640</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4">
         <v>6</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ENTORNO CONSULTORIA, DISEÑO Y SERVICIOS AMBIENTALES SAS</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>328947369.0526316</v>
-      </c>
-      <c r="E4" t="n">
-        <v>62500000.12</v>
-      </c>
-      <c r="F4" t="n">
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4">
+        <v>328947369.05263162</v>
+      </c>
+      <c r="E4">
+        <v>62500000.119999997</v>
+      </c>
+      <c r="F4">
         <v>391447369</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>901852866</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5">
         <v>5</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>EMPRESA DE DESARROLLO TERRITORIAL DE DONMATÍAS S.A.S.</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5">
         <v>82845580</v>
       </c>
-      <c r="E5" t="n">
-        <v>15740660.2</v>
-      </c>
-      <c r="F5" t="n">
+      <c r="E5">
+        <v>15740660.199999999</v>
+      </c>
+      <c r="F5">
         <v>98586240</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor return and excluded expense calculations; update utility types for consistency
</commit_message>
<xml_diff>
--- a/consolidado_exogena.xlsx
+++ b/consolidado_exogena.xlsx
@@ -8,19 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acuerdode-my.sharepoint.com/personal/sistemas_eso_gov_co/Documents/Preparador de exogenas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_2B59F87F11DFCA2F158BC0F34C1510344D07F1B2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB9CA89E-D6A6-4103-8034-104691F1B399}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_3161D90AA501063700A38834E7D8AA9AD75A1B37" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACBE0A51-2B28-40E0-BCB2-E6140F9D4C42}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ingresos" sheetId="1" r:id="rId1"/>
+    <sheet name="Notas Crédito" sheetId="2" r:id="rId2"/>
+    <sheet name="Devoluciones" sheetId="3" r:id="rId3"/>
+    <sheet name="Gastos" sheetId="4" r:id="rId4"/>
+    <sheet name="Gastos Excluidos" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="24">
   <si>
     <t>NIT Receptor</t>
   </si>
@@ -50,6 +54,48 @@
   </si>
   <si>
     <t>EMPRESA DE DESARROLLO TERRITORIAL DE DONMATÍAS S.A.S.</t>
+  </si>
+  <si>
+    <t>NIT Emisor</t>
+  </si>
+  <si>
+    <t>Nombre Emisor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carlos Alberto Restrepo Osorio </t>
+  </si>
+  <si>
+    <t>ELECTRICOS ITAGUI S.A.S</t>
+  </si>
+  <si>
+    <t>KKONG SAS</t>
+  </si>
+  <si>
+    <t>JULIETTE ALEXANDRA ACEVEDO LOPEZ</t>
+  </si>
+  <si>
+    <t>Comercial Modelo S.A.S</t>
+  </si>
+  <si>
+    <t>COMPEL S.A</t>
+  </si>
+  <si>
+    <t>BAZAR AMERICANO S.A.S</t>
+  </si>
+  <si>
+    <t>ALMACEN EL CONSTRUCTOR BOLIVAR SA</t>
+  </si>
+  <si>
+    <t>INVESA S.A</t>
+  </si>
+  <si>
+    <t>JURIS.MARCA SAS</t>
+  </si>
+  <si>
+    <t>CAMARA DE COMERCIO DE MEDELLIN PARA ANTIOQUIA</t>
+  </si>
+  <si>
+    <t>SOLUCIONES ALEGRA S.A.S</t>
   </si>
 </sst>
 </file>
@@ -393,9 +439,9 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="3.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="55.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="57.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
   </cols>
@@ -503,4 +549,478 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr codeName="Hoja2"/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>860006522</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2">
+        <v>520000</v>
+      </c>
+      <c r="E2">
+        <v>98800</v>
+      </c>
+      <c r="F2">
+        <v>698800</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr codeName="Hoja3"/>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>70557710</v>
+      </c>
+      <c r="B2">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2">
+        <v>861500</v>
+      </c>
+      <c r="E2">
+        <v>163685</v>
+      </c>
+      <c r="F2">
+        <v>1025185</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>900165621</v>
+      </c>
+      <c r="B3">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3">
+        <v>11092.42105263158</v>
+      </c>
+      <c r="E3">
+        <v>2107.56</v>
+      </c>
+      <c r="F3">
+        <v>13200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>901456163</v>
+      </c>
+      <c r="B4">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4">
+        <v>12605040</v>
+      </c>
+      <c r="E4">
+        <v>2394957.6</v>
+      </c>
+      <c r="F4">
+        <v>14999997.6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr codeName="Hoja4"/>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>43180997</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2">
+        <v>175798.68421052629</v>
+      </c>
+      <c r="E2">
+        <v>33401.75</v>
+      </c>
+      <c r="F2">
+        <v>209200.44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>70557710</v>
+      </c>
+      <c r="B3">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3">
+        <v>1745900</v>
+      </c>
+      <c r="E3">
+        <v>331721</v>
+      </c>
+      <c r="F3">
+        <v>2077621</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>800002026</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4">
+        <v>4205042</v>
+      </c>
+      <c r="E4">
+        <v>798957.98</v>
+      </c>
+      <c r="F4">
+        <v>5004000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>800147520</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5">
+        <v>114950</v>
+      </c>
+      <c r="E5">
+        <v>21840.5</v>
+      </c>
+      <c r="F5">
+        <v>136791</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>800149246</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>571462.21052631584</v>
+      </c>
+      <c r="E6">
+        <v>108577.82</v>
+      </c>
+      <c r="F6">
+        <v>680040.02</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>811037574</v>
+      </c>
+      <c r="B7">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7">
+        <v>880672.21052631573</v>
+      </c>
+      <c r="E7">
+        <v>167327.72</v>
+      </c>
+      <c r="F7">
+        <v>1048000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>890900652</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8">
+        <v>1818991.631578947</v>
+      </c>
+      <c r="E8">
+        <v>345608.41</v>
+      </c>
+      <c r="F8">
+        <v>2164600.04</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>900165621</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9">
+        <v>818873.42105263157</v>
+      </c>
+      <c r="E9">
+        <v>155585.95000000001</v>
+      </c>
+      <c r="F9">
+        <v>974459.4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>901016781</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10">
+        <v>230084.05263157899</v>
+      </c>
+      <c r="E10">
+        <v>43715.97</v>
+      </c>
+      <c r="F10">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>901456163</v>
+      </c>
+      <c r="B11">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11">
+        <v>395084135.42105258</v>
+      </c>
+      <c r="E11">
+        <v>75065985.730000004</v>
+      </c>
+      <c r="F11">
+        <v>470150121.14999998</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <sheetPr codeName="Hoja5"/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="49" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>890905080</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>680300</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>900559088</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>2059000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>